<commit_message>
final attempt at improving the prediction accuracy
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1077,54 +1077,54 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>43053</v>
+        <v>85576</v>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C2" t="b">
         <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A♯/B♭</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.569</v>
+        <v>0.595</v>
       </c>
       <c r="H2" t="n">
-        <v>0.264</v>
+        <v>0.836</v>
       </c>
       <c r="I2" t="n">
-        <v>-13.198</v>
+        <v>-6.622</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0312</v>
+        <v>0.0398</v>
       </c>
       <c r="K2" t="n">
-        <v>0.776</v>
+        <v>0.00689</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>4.39e-06</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0.165</v>
+        <v>0.34</v>
       </c>
       <c r="O2" t="n">
-        <v>0.31</v>
+        <v>0.441</v>
       </c>
       <c r="P2" t="n">
-        <v>112.866</v>
+        <v>116</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -1163,362 +1163,362 @@
         <v>0</v>
       </c>
       <c r="AC2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CS2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CT2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CU2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CV2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CX2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CY2" t="b">
+        <v>0</v>
+      </c>
+      <c r="CZ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DA2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DC2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DD2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DF2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DH2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DI2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DK2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DM2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DN2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DO2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DP2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DQ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DR2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DS2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DT2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DU2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DV2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DW2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DX2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DY2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DZ2" t="b">
         <v>1</v>
-      </c>
-      <c r="AD2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AY2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CS2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CT2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CU2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CV2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CW2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CX2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CY2" t="b">
-        <v>0</v>
-      </c>
-      <c r="CZ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DA2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DB2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DC2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DD2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DE2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DG2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DH2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DI2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DK2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DL2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DM2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DO2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DP2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DQ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DS2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DT2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DU2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DV2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DW2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DX2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DY2" t="b">
-        <v>0</v>
-      </c>
-      <c r="DZ2" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>86278</v>
+        <v>62669</v>
       </c>
       <c r="B3" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>3.2</v>
+        <v>5.2</v>
       </c>
       <c r="G3" t="n">
-        <v>0.287</v>
+        <v>0.455</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0808</v>
+        <v>0.978</v>
       </c>
       <c r="I3" t="n">
-        <v>-21.822</v>
+        <v>-3.009</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0496</v>
+        <v>0.163</v>
       </c>
       <c r="K3" t="n">
-        <v>0.916</v>
+        <v>0.00744</v>
       </c>
       <c r="L3" t="n">
-        <v>0.312</v>
+        <v>0.0044</v>
       </c>
       <c r="M3" t="n">
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.121</v>
+        <v>0.329</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0588</v>
+        <v>0.543</v>
       </c>
       <c r="P3" t="n">
-        <v>62.194</v>
+        <v>189.958</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -1704,7 +1704,7 @@
         <v>0</v>
       </c>
       <c r="BZ3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CA3" t="b">
         <v>0</v>
@@ -1860,59 +1860,59 @@
         <v>0</v>
       </c>
       <c r="DZ3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>50963</v>
+        <v>58184</v>
       </c>
       <c r="B4" t="n">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="C4" t="b">
         <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C♯/D♭</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>3.4</v>
       </c>
       <c r="G4" t="n">
-        <v>0.792</v>
+        <v>0.367</v>
       </c>
       <c r="H4" t="n">
-        <v>0.895</v>
+        <v>0.893</v>
       </c>
       <c r="I4" t="n">
-        <v>-3.112</v>
+        <v>-3.631</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0589</v>
+        <v>0.06279999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>0.165</v>
+        <v>0.049</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>8.420000000000001e-06</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0501</v>
+        <v>0.178</v>
       </c>
       <c r="O4" t="n">
-        <v>0.794</v>
+        <v>0.805</v>
       </c>
       <c r="P4" t="n">
-        <v>94.968</v>
+        <v>79.80800000000001</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -1975,265 +1975,265 @@
         <v>0</v>
       </c>
       <c r="AK4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CS4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CT4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CU4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CV4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CX4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CY4" t="b">
+        <v>0</v>
+      </c>
+      <c r="CZ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DC4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DD4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DF4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DG4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DH4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DI4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DJ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DK4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DL4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DM4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DN4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DO4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DP4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DQ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DR4" t="b">
+        <v>0</v>
+      </c>
+      <c r="DS4" t="b">
         <v>1</v>
-      </c>
-      <c r="AL4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AY4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BE4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY4" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF4" t="b">
-        <v>1</v>
-      </c>
-      <c r="CG4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CR4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CS4" t="b">
-        <v>1</v>
-      </c>
-      <c r="CT4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CU4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CV4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CW4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CX4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CY4" t="b">
-        <v>0</v>
-      </c>
-      <c r="CZ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DA4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DB4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DC4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DD4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DE4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DF4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DG4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DH4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DI4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DJ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DK4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DL4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DM4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DN4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DO4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DP4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DQ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DR4" t="b">
-        <v>0</v>
-      </c>
-      <c r="DS4" t="b">
-        <v>0</v>
       </c>
       <c r="DT4" t="b">
         <v>0</v>
@@ -2259,54 +2259,54 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>80991</v>
+        <v>51961</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="C5" t="b">
         <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>0.669</v>
+        <v>0.582</v>
       </c>
       <c r="H5" t="n">
-        <v>0.552</v>
+        <v>0.64</v>
       </c>
       <c r="I5" t="n">
-        <v>-7.98</v>
+        <v>-7.586</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0587</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.317</v>
       </c>
       <c r="L5" t="n">
-        <v>0.000874</v>
+        <v>0.178</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="N5" t="n">
-        <v>0.321</v>
+        <v>0.268</v>
       </c>
       <c r="O5" t="n">
-        <v>0.488</v>
+        <v>0.266</v>
       </c>
       <c r="P5" t="n">
-        <v>100.102</v>
+        <v>199.981</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -2366,19 +2366,19 @@
         <v>0</v>
       </c>
       <c r="AJ5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN5" t="b">
         <v>1</v>
-      </c>
-      <c r="AK5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN5" t="b">
-        <v>0</v>
       </c>
       <c r="AO5" t="b">
         <v>0</v>
@@ -2653,54 +2653,54 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>84141</v>
+        <v>47451</v>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C6" t="b">
         <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>2.6</v>
+        <v>4.7</v>
       </c>
       <c r="G6" t="n">
-        <v>0.787</v>
+        <v>0.243</v>
       </c>
       <c r="H6" t="n">
-        <v>0.36</v>
+        <v>0.619</v>
       </c>
       <c r="I6" t="n">
-        <v>-9.374000000000001</v>
+        <v>-6.287</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0649</v>
+        <v>0.0336</v>
       </c>
       <c r="K6" t="n">
-        <v>0.831</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>0.31</v>
+        <v>5e-06</v>
       </c>
       <c r="M6" t="n">
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0.101</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.894</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="P6" t="n">
-        <v>140.268</v>
+        <v>143.609</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -2823,7 +2823,7 @@
         <v>0</v>
       </c>
       <c r="BE6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF6" t="b">
         <v>0</v>
@@ -3027,7 +3027,7 @@
         <v>0</v>
       </c>
       <c r="DU6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DV6" t="b">
         <v>0</v>
@@ -3047,7 +3047,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>11998</v>
+        <v>30991</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -3061,40 +3061,40 @@
         </is>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>2.7</v>
+        <v>4.4</v>
       </c>
       <c r="G7" t="n">
-        <v>0.754</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>0.763</v>
+        <v>0.457</v>
       </c>
       <c r="I7" t="n">
-        <v>-4.627</v>
+        <v>-10.013</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0435</v>
+        <v>0.0374</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0301</v>
+        <v>0.66</v>
       </c>
       <c r="L7" t="n">
-        <v>2.23e-05</v>
+        <v>0.0391</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0901</v>
+        <v>0.181</v>
       </c>
       <c r="O7" t="n">
-        <v>0.464</v>
+        <v>0.418</v>
       </c>
       <c r="P7" t="n">
-        <v>117.953</v>
+        <v>122.518</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -3124,7 +3124,7 @@
         <v>0</v>
       </c>
       <c r="Z7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA7" t="b">
         <v>0</v>
@@ -3157,209 +3157,209 @@
         <v>0</v>
       </c>
       <c r="AK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AY7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM7" t="b">
         <v>1</v>
       </c>
-      <c r="AL7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU7" t="b">
+      <c r="CN7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CS7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CT7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CU7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CV7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CX7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CY7" t="b">
+        <v>0</v>
+      </c>
+      <c r="CZ7" t="b">
         <v>1</v>
       </c>
-      <c r="AV7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AY7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BE7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR7" t="b">
-        <v>1</v>
-      </c>
-      <c r="BS7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY7" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CR7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CS7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CT7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CU7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CV7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CW7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CX7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CY7" t="b">
-        <v>0</v>
-      </c>
-      <c r="CZ7" t="b">
-        <v>0</v>
-      </c>
       <c r="DA7" t="b">
         <v>0</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>0</v>
       </c>
       <c r="DW7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DX7" t="b">
         <v>0</v>
@@ -3441,54 +3441,54 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>72775</v>
+        <v>12198</v>
       </c>
       <c r="B8" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E8" t="b">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>3.1</v>
+        <v>4.1</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.385</v>
       </c>
       <c r="H8" t="n">
-        <v>0.845</v>
+        <v>0.719</v>
       </c>
       <c r="I8" t="n">
-        <v>-4.236</v>
+        <v>-5.493</v>
       </c>
       <c r="J8" t="n">
-        <v>0.0362</v>
+        <v>0.186</v>
       </c>
       <c r="K8" t="n">
-        <v>0.00757</v>
+        <v>0.446</v>
       </c>
       <c r="L8" t="n">
-        <v>3.66e-05</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.115</v>
+        <v>0.111</v>
       </c>
       <c r="O8" t="n">
-        <v>0.262</v>
+        <v>0.646</v>
       </c>
       <c r="P8" t="n">
-        <v>91.98</v>
+        <v>87.495</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -3515,38 +3515,38 @@
         <v>0</v>
       </c>
       <c r="Y8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="b">
         <v>1</v>
       </c>
-      <c r="Z8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI8" t="b">
-        <v>0</v>
-      </c>
       <c r="AJ8" t="b">
         <v>0</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>0</v>
       </c>
       <c r="BL8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM8" t="b">
         <v>0</v>
@@ -3835,10 +3835,10 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>41898</v>
+        <v>19100</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C9" t="b">
         <v>0</v>
@@ -3852,37 +3852,37 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="G9" t="n">
-        <v>0.524</v>
+        <v>0.534</v>
       </c>
       <c r="H9" t="n">
-        <v>0.739</v>
+        <v>0.592</v>
       </c>
       <c r="I9" t="n">
-        <v>-6.681</v>
+        <v>-8.56</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0386</v>
+        <v>0.0352</v>
       </c>
       <c r="K9" t="n">
-        <v>0.215</v>
+        <v>0.0426</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.0385</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="N9" t="n">
-        <v>0.0636</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="O9" t="n">
-        <v>0.48</v>
+        <v>0.202</v>
       </c>
       <c r="P9" t="n">
-        <v>83.095</v>
+        <v>88.012</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4095,7 +4095,7 @@
         <v>0</v>
       </c>
       <c r="CI9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CJ9" t="b">
         <v>0</v>
@@ -4194,7 +4194,7 @@
         <v>0</v>
       </c>
       <c r="DP9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DQ9" t="b">
         <v>0</v>
@@ -4229,390 +4229,390 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>83993</v>
+        <v>72918</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>F♯/G♭</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-4.78</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.0009859999999999999</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="P10" t="n">
+        <v>191.86</v>
+      </c>
+      <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
+        <v>0</v>
+      </c>
+      <c r="S10" t="b">
+        <v>0</v>
+      </c>
+      <c r="T10" t="b">
+        <v>0</v>
+      </c>
+      <c r="U10" t="b">
+        <v>0</v>
+      </c>
+      <c r="V10" t="b">
+        <v>0</v>
+      </c>
+      <c r="W10" t="b">
+        <v>0</v>
+      </c>
+      <c r="X10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CS10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CT10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CU10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CV10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CX10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CY10" t="b">
+        <v>0</v>
+      </c>
+      <c r="CZ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DB10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DC10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DD10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DE10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DF10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DG10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DH10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DI10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DJ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DK10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DM10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DN10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DO10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DP10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DQ10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DR10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DS10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DT10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DU10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DV10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DW10" t="b">
+        <v>0</v>
+      </c>
+      <c r="DX10" t="b">
         <v>1</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E10" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.631</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-4.179</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.101</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.107</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.373</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.782</v>
-      </c>
-      <c r="P10" t="n">
-        <v>156.941</v>
-      </c>
-      <c r="Q10" t="b">
-        <v>0</v>
-      </c>
-      <c r="R10" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10" t="b">
-        <v>0</v>
-      </c>
-      <c r="T10" t="b">
-        <v>0</v>
-      </c>
-      <c r="U10" t="b">
-        <v>0</v>
-      </c>
-      <c r="V10" t="b">
-        <v>0</v>
-      </c>
-      <c r="W10" t="b">
-        <v>0</v>
-      </c>
-      <c r="X10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AY10" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BE10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY10" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ10" t="b">
-        <v>1</v>
-      </c>
-      <c r="CR10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CS10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CT10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CU10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CV10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CW10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CX10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CY10" t="b">
-        <v>0</v>
-      </c>
-      <c r="CZ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DA10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DB10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DC10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DD10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DE10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DF10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DG10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DH10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DI10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DJ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DK10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DL10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DM10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DN10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DO10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DP10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DQ10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DR10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DS10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DT10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DU10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DV10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DW10" t="b">
-        <v>0</v>
-      </c>
-      <c r="DX10" t="b">
-        <v>0</v>
       </c>
       <c r="DY10" t="b">
         <v>0</v>
@@ -4623,54 +4623,54 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>77041</v>
+        <v>3056</v>
       </c>
       <c r="B11" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="C11" t="b">
         <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E11" t="b">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>3.2</v>
+        <v>5.4</v>
       </c>
       <c r="G11" t="n">
-        <v>0.305</v>
+        <v>0.257</v>
       </c>
       <c r="H11" t="n">
-        <v>0.847</v>
+        <v>0.221</v>
       </c>
       <c r="I11" t="n">
-        <v>-8.75</v>
+        <v>-9.013999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0638</v>
+        <v>0.0302</v>
       </c>
       <c r="K11" t="n">
-        <v>0.00559</v>
+        <v>0.882</v>
       </c>
       <c r="L11" t="n">
-        <v>2.79e-06</v>
+        <v>0.00175</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.52</v>
+        <v>0.608</v>
       </c>
       <c r="O11" t="n">
-        <v>0.48</v>
+        <v>0.361</v>
       </c>
       <c r="P11" t="n">
-        <v>133.952</v>
+        <v>144.96</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -4796,7 +4796,7 @@
         <v>0</v>
       </c>
       <c r="BF11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG11" t="b">
         <v>0</v>
@@ -4823,175 +4823,175 @@
         <v>0</v>
       </c>
       <c r="BO11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CS11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CT11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CU11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CV11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CX11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CY11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CZ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DB11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DC11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DD11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DE11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DF11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DG11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DH11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DI11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DJ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DM11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DN11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DO11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="DS11" t="b">
         <v>1</v>
-      </c>
-      <c r="BP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CS11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CT11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CU11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CV11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CW11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CX11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CY11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CZ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DA11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DB11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DC11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DD11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DE11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DF11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DG11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DH11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DI11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DJ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DM11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DN11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DO11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="DS11" t="b">
-        <v>0</v>
       </c>
       <c r="DT11" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
final tweaks to workbook
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -1077,54 +1077,54 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>85576</v>
+        <v>38288</v>
       </c>
       <c r="B2" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C2" t="b">
         <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D♯/E♭</t>
         </is>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.595</v>
+        <v>0.627</v>
       </c>
       <c r="H2" t="n">
-        <v>0.836</v>
+        <v>0.527</v>
       </c>
       <c r="I2" t="n">
-        <v>-6.622</v>
+        <v>-5.78</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0398</v>
+        <v>0.0315</v>
       </c>
       <c r="K2" t="n">
-        <v>0.00689</v>
+        <v>0.406</v>
       </c>
       <c r="L2" t="n">
-        <v>4.39e-06</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0.34</v>
+        <v>0.161</v>
       </c>
       <c r="O2" t="n">
-        <v>0.441</v>
+        <v>0.433</v>
       </c>
       <c r="P2" t="n">
-        <v>116</v>
+        <v>117.895</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -1247,7 +1247,7 @@
         <v>0</v>
       </c>
       <c r="BE2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BF2" t="b">
         <v>0</v>
@@ -1466,59 +1466,59 @@
         <v>0</v>
       </c>
       <c r="DZ2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>62669</v>
+        <v>72397</v>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>A♯/B♭</t>
         </is>
       </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>5.2</v>
+        <v>3.7</v>
       </c>
       <c r="G3" t="n">
-        <v>0.455</v>
+        <v>0.536</v>
       </c>
       <c r="H3" t="n">
-        <v>0.978</v>
+        <v>0.399</v>
       </c>
       <c r="I3" t="n">
-        <v>-3.009</v>
+        <v>-7.579</v>
       </c>
       <c r="J3" t="n">
-        <v>0.163</v>
+        <v>0.0319</v>
       </c>
       <c r="K3" t="n">
-        <v>0.00744</v>
+        <v>0.307</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0044</v>
+        <v>0.000327</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.329</v>
+        <v>0.105</v>
       </c>
       <c r="O3" t="n">
-        <v>0.543</v>
+        <v>0.476</v>
       </c>
       <c r="P3" t="n">
-        <v>189.958</v>
+        <v>81.371</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -1548,7 +1548,7 @@
         <v>0</v>
       </c>
       <c r="Z3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA3" t="b">
         <v>0</v>
@@ -1662,7 +1662,7 @@
         <v>0</v>
       </c>
       <c r="BL3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM3" t="b">
         <v>0</v>
@@ -1704,47 +1704,47 @@
         <v>0</v>
       </c>
       <c r="BZ3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL3" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM3" t="b">
         <v>1</v>
       </c>
-      <c r="CA3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL3" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM3" t="b">
-        <v>0</v>
-      </c>
       <c r="CN3" t="b">
         <v>0</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>0</v>
       </c>
       <c r="CZ3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DA3" t="b">
         <v>0</v>
@@ -1865,10 +1865,10 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>58184</v>
+        <v>44181</v>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C4" t="b">
         <v>0</v>
@@ -1879,116 +1879,116 @@
         </is>
       </c>
       <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-12.147</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.0362</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.717</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="P4" t="n">
+        <v>148.093</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" t="b">
+        <v>0</v>
+      </c>
+      <c r="V4" t="b">
+        <v>0</v>
+      </c>
+      <c r="W4" t="b">
+        <v>0</v>
+      </c>
+      <c r="X4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.367</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.893</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-3.631</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.06279999999999999</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="L4" t="n">
-        <v>8.420000000000001e-06</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.805</v>
-      </c>
-      <c r="P4" t="n">
-        <v>79.80800000000001</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4" t="b">
-        <v>0</v>
-      </c>
-      <c r="S4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4" t="b">
-        <v>0</v>
-      </c>
-      <c r="U4" t="b">
-        <v>0</v>
-      </c>
-      <c r="V4" t="b">
-        <v>0</v>
-      </c>
-      <c r="W4" t="b">
-        <v>0</v>
-      </c>
-      <c r="X4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO4" t="b">
-        <v>0</v>
-      </c>
       <c r="AP4" t="b">
         <v>0</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>0</v>
       </c>
       <c r="DS4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DT4" t="b">
         <v>0</v>
@@ -2259,10 +2259,10 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>51961</v>
+        <v>51446</v>
       </c>
       <c r="B5" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C5" t="b">
         <v>0</v>
@@ -2276,37 +2276,37 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="G5" t="n">
-        <v>0.582</v>
+        <v>0.473</v>
       </c>
       <c r="H5" t="n">
-        <v>0.64</v>
+        <v>0.575</v>
       </c>
       <c r="I5" t="n">
-        <v>-7.586</v>
+        <v>-9.477</v>
       </c>
       <c r="J5" t="n">
-        <v>0.09619999999999999</v>
+        <v>0.348</v>
       </c>
       <c r="K5" t="n">
-        <v>0.317</v>
+        <v>0.316</v>
       </c>
       <c r="L5" t="n">
-        <v>0.178</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.268</v>
+        <v>0.105</v>
       </c>
       <c r="O5" t="n">
-        <v>0.266</v>
+        <v>0.529</v>
       </c>
       <c r="P5" t="n">
-        <v>199.981</v>
+        <v>81.251</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -2378,55 +2378,55 @@
         <v>0</v>
       </c>
       <c r="AN5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB5" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC5" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="b">
         <v>1</v>
-      </c>
-      <c r="AO5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AY5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD5" t="b">
-        <v>0</v>
       </c>
       <c r="BE5" t="b">
         <v>0</v>
@@ -2653,54 +2653,54 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>47451</v>
+        <v>53937</v>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C6" t="b">
         <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G♯/A♭</t>
         </is>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>4.7</v>
+        <v>1.8</v>
       </c>
       <c r="G6" t="n">
-        <v>0.243</v>
+        <v>0.29</v>
       </c>
       <c r="H6" t="n">
-        <v>0.619</v>
+        <v>0.0372</v>
       </c>
       <c r="I6" t="n">
-        <v>-6.287</v>
+        <v>-17.504</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0336</v>
+        <v>0.0415</v>
       </c>
       <c r="K6" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>5e-06</v>
+        <v>0.918</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>0.92</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.23</v>
       </c>
       <c r="O6" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.197</v>
       </c>
       <c r="P6" t="n">
-        <v>143.609</v>
+        <v>82.14100000000001</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -2823,49 +2823,49 @@
         <v>0</v>
       </c>
       <c r="BE6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS6" t="b">
         <v>1</v>
-      </c>
-      <c r="BF6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR6" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS6" t="b">
-        <v>0</v>
       </c>
       <c r="BT6" t="b">
         <v>0</v>
@@ -3047,54 +3047,54 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>30991</v>
+        <v>485</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C7" t="b">
         <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>G♯/A♭</t>
         </is>
       </c>
       <c r="E7" t="b">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.68</v>
       </c>
       <c r="H7" t="n">
-        <v>0.457</v>
+        <v>0.154</v>
       </c>
       <c r="I7" t="n">
-        <v>-10.013</v>
+        <v>-20.01</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0374</v>
+        <v>0.0407</v>
       </c>
       <c r="K7" t="n">
-        <v>0.66</v>
+        <v>0.975</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0391</v>
+        <v>0.824</v>
       </c>
       <c r="M7" t="n">
-        <v>0.04</v>
+        <v>0.82</v>
       </c>
       <c r="N7" t="n">
-        <v>0.181</v>
+        <v>0.114</v>
       </c>
       <c r="O7" t="n">
-        <v>0.418</v>
+        <v>0.149</v>
       </c>
       <c r="P7" t="n">
-        <v>122.518</v>
+        <v>120.076</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -3124,59 +3124,59 @@
         <v>0</v>
       </c>
       <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="b">
         <v>1</v>
       </c>
-      <c r="AA7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP7" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ7" t="b">
-        <v>0</v>
-      </c>
       <c r="AR7" t="b">
         <v>0</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>0</v>
       </c>
       <c r="CM7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CN7" t="b">
         <v>0</v>
@@ -3358,7 +3358,7 @@
         <v>0</v>
       </c>
       <c r="CZ7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DA7" t="b">
         <v>0</v>
@@ -3441,39 +3441,39 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>12198</v>
+        <v>31278</v>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E8" t="b">
         <v>1</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="E8" t="b">
-        <v>0</v>
-      </c>
       <c r="F8" t="n">
-        <v>4.1</v>
+        <v>2.7</v>
       </c>
       <c r="G8" t="n">
-        <v>0.385</v>
+        <v>0.821</v>
       </c>
       <c r="H8" t="n">
-        <v>0.719</v>
+        <v>0.644</v>
       </c>
       <c r="I8" t="n">
-        <v>-5.493</v>
+        <v>-7.435</v>
       </c>
       <c r="J8" t="n">
-        <v>0.186</v>
+        <v>0.133</v>
       </c>
       <c r="K8" t="n">
-        <v>0.446</v>
+        <v>0.229</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -3482,13 +3482,13 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.111</v>
+        <v>0.0806</v>
       </c>
       <c r="O8" t="n">
-        <v>0.646</v>
+        <v>0.93</v>
       </c>
       <c r="P8" t="n">
-        <v>87.495</v>
+        <v>134.961</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -3545,187 +3545,187 @@
         <v>0</v>
       </c>
       <c r="AI8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AY8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AZ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BB8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BC8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BD8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BE8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP8" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ8" t="b">
         <v>1</v>
-      </c>
-      <c r="AJ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AY8" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BE8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY8" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP8" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ8" t="b">
-        <v>0</v>
       </c>
       <c r="CR8" t="b">
         <v>0</v>
@@ -3835,54 +3835,54 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>19100</v>
+        <v>74476</v>
       </c>
       <c r="B9" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C9" t="b">
         <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="G9" t="n">
-        <v>0.534</v>
+        <v>0.264</v>
       </c>
       <c r="H9" t="n">
-        <v>0.592</v>
+        <v>0.0224</v>
       </c>
       <c r="I9" t="n">
-        <v>-8.56</v>
+        <v>-29.738</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0352</v>
+        <v>0.0374</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0426</v>
+        <v>0.968</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0385</v>
+        <v>0.887</v>
       </c>
       <c r="M9" t="n">
-        <v>0.04</v>
+        <v>0.89</v>
       </c>
       <c r="N9" t="n">
-        <v>0.09569999999999999</v>
+        <v>0.103</v>
       </c>
       <c r="O9" t="n">
-        <v>0.202</v>
+        <v>0.266</v>
       </c>
       <c r="P9" t="n">
-        <v>88.012</v>
+        <v>54.356</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -4095,34 +4095,34 @@
         <v>0</v>
       </c>
       <c r="CI9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ9" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR9" t="b">
         <v>1</v>
-      </c>
-      <c r="CJ9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ9" t="b">
-        <v>0</v>
-      </c>
-      <c r="CR9" t="b">
-        <v>0</v>
       </c>
       <c r="CS9" t="b">
         <v>0</v>
@@ -4229,54 +4229,54 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>72918</v>
+        <v>82853</v>
       </c>
       <c r="B10" t="n">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="C10" t="b">
         <v>0</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>F♯/G♭</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E10" t="b">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
       <c r="G10" t="n">
-        <v>0.626</v>
+        <v>0.405</v>
       </c>
       <c r="H10" t="n">
-        <v>0.617</v>
+        <v>0.257</v>
       </c>
       <c r="I10" t="n">
-        <v>-4.78</v>
+        <v>-16.123</v>
       </c>
       <c r="J10" t="n">
-        <v>0.275</v>
+        <v>0.031</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0111</v>
+        <v>0.948</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0009859999999999999</v>
+        <v>0.879</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="N10" t="n">
-        <v>0.212</v>
+        <v>0.0941</v>
       </c>
       <c r="O10" t="n">
-        <v>0.425</v>
+        <v>0.332</v>
       </c>
       <c r="P10" t="n">
-        <v>191.86</v>
+        <v>153.389</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -4603,7 +4603,7 @@
         <v>0</v>
       </c>
       <c r="DU10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DV10" t="b">
         <v>0</v>
@@ -4612,7 +4612,7 @@
         <v>0</v>
       </c>
       <c r="DX10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DY10" t="b">
         <v>0</v>
@@ -4623,157 +4623,157 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>3056</v>
+        <v>8993</v>
       </c>
       <c r="B11" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C11" t="b">
         <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E11" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-5.848</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.000168</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.428</v>
+      </c>
+      <c r="P11" t="n">
+        <v>164.076</v>
+      </c>
+      <c r="Q11" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" t="b">
+        <v>0</v>
+      </c>
+      <c r="S11" t="b">
+        <v>0</v>
+      </c>
+      <c r="T11" t="b">
+        <v>0</v>
+      </c>
+      <c r="U11" t="b">
+        <v>0</v>
+      </c>
+      <c r="V11" t="b">
+        <v>0</v>
+      </c>
+      <c r="W11" t="b">
+        <v>0</v>
+      </c>
+      <c r="X11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AT11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AW11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AX11" t="b">
         <v>1</v>
       </c>
-      <c r="F11" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.257</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.221</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-9.013999999999999</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.0302</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.882</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.00175</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.608</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.361</v>
-      </c>
-      <c r="P11" t="n">
-        <v>144.96</v>
-      </c>
-      <c r="Q11" t="b">
-        <v>0</v>
-      </c>
-      <c r="R11" t="b">
-        <v>0</v>
-      </c>
-      <c r="S11" t="b">
-        <v>0</v>
-      </c>
-      <c r="T11" t="b">
-        <v>0</v>
-      </c>
-      <c r="U11" t="b">
-        <v>0</v>
-      </c>
-      <c r="V11" t="b">
-        <v>0</v>
-      </c>
-      <c r="W11" t="b">
-        <v>0</v>
-      </c>
-      <c r="X11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX11" t="b">
-        <v>0</v>
-      </c>
       <c r="AY11" t="b">
         <v>0</v>
       </c>
@@ -4796,143 +4796,143 @@
         <v>0</v>
       </c>
       <c r="BF11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BI11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BO11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BS11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BT11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BU11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BV11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BW11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BX11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BY11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BZ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CB11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CD11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CE11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CF11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CG11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CH11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CI11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CJ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CK11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CM11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CN11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CO11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CP11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CQ11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CR11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CS11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CT11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CU11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CV11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CW11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CX11" t="b">
+        <v>0</v>
+      </c>
+      <c r="CY11" t="b">
         <v>1</v>
       </c>
-      <c r="BG11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BO11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BS11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BT11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BU11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BV11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BW11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BX11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BY11" t="b">
-        <v>0</v>
-      </c>
-      <c r="BZ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CA11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CB11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CC11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CD11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CE11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CF11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CG11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CH11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CI11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CJ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CK11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CL11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CM11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CN11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CO11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CP11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CQ11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CR11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CS11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CT11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CU11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CV11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CW11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CX11" t="b">
-        <v>0</v>
-      </c>
-      <c r="CY11" t="b">
-        <v>0</v>
-      </c>
       <c r="CZ11" t="b">
         <v>0</v>
       </c>
@@ -4991,7 +4991,7 @@
         <v>0</v>
       </c>
       <c r="DS11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DT11" t="b">
         <v>0</v>

</xml_diff>